<commit_message>
Keep embedded photos fully inside their cells: wider photo column, smaller centered images
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FqYowjsZP867X3muhU5EDZ
</commit_message>
<xml_diff>
--- a/gear-study/Gear_Inventory_GoogleSheets.xlsx
+++ b/gear-study/Gear_Inventory_GoogleSheets.xlsx
@@ -578,7 +578,7 @@
   <dimension ref="A1:O321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
@@ -21751,7 +21751,7 @@
   <dimension ref="A1:O75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
@@ -26729,7 +26729,7 @@
   <dimension ref="A1:O75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
@@ -31804,7 +31804,7 @@
   <dimension ref="A1:O47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
@@ -34956,7 +34956,7 @@
   <dimension ref="A1:O127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>

</xml_diff>